<commit_message>
Feat: Update Formulario_Salida_Vitalis.xlsx with new data
</commit_message>
<xml_diff>
--- a/data/input/Formulario_Salida_Vitalis.xlsx
+++ b/data/input/Formulario_Salida_Vitalis.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias_Clinicas_Entrada" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulario_Salida" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historias_Clinicas_Entrada" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Formulario_Salida" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1092,6 +1092,117 @@
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Paciente Mateo Alejandro Buitrago, CC 1.032.667.410, reside en Cra 20 #33-05, Bogotá, tel. 302-555-0222, 19 años. Consulta traído por su familia, quienes refieren cambios de comportamiento, aislamiento social y bajo rendimiento académico en el último semestre. El paciente reconoce consumo frecuente de marihuana (diario) desde hace 8 meses, y fuma cigarrillo ocasionalmente. Niega otras sustancias. Sin antecedentes médicos previos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>REG-13</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Diego Fernando Salazar Prieto</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>1.045.223.887</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Cra 68 #24-10, Bogotá</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>305-555-0233</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Paciente Diego Fernando Salazar Prieto, CC 1.045.223.887, reside en Cra 68 #24-10, Bogotá, tel. 305-555-0233, 31 años. Consulta por cefalea pulsátil hemicraneal derecha de 8 horas de evolución, acompañada de náuseas, vómito y fotofobia intensa. Antecedente de migraña en el padre. No fuma. Niega consumo de sustancias. Episodios similares recurrentes desde hace 3 años, 2-3 veces al mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>REG-14</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Mónica Alexandra Duarte Peña</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>52.667.910</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Calle 94 #15-40, Bogotá</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>311-555-0244</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Paciente Mónica Alexandra Duarte Peña, CC 52.667.910, domicilio Calle 94 #15-40, Bogotá, tel. 311-555-0244, 49 años. Consulta de control, cifras de presión arterial 168/104 mmHg en tres tomas consecutivas, pese a tratamiento con enalapril. Refiere cefalea occipital matutina ocasional. No fuma. Niega consumo de sustancias. Antecedente de dislipidemia y madre con hipertensión arterial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>REG-15</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Andrés Camilo Vargas Niño</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>1.098.334.520</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Cra 30 #45-12, Cali</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>318-555-0255</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Paciente Andrés Camilo Vargas Niño, CC 1.098.334.520, dirección Cra 30 #45-12, Cali, tel. 318-555-0255, 24 años. Consulta por dolor abdominal que inició periumbilical y migró a fosa ilíaca derecha en las últimas 12 horas, con fiebre de 38.4°C, náuseas y signo de rebote positivo (Blumberg positivo) en el examen físico. Leucocitosis de 14.200/mm³ con desviación izquierda. No fuma. Niega consumo de sustancias. Sin antecedentes médicos relevantes.</t>
         </is>
       </c>
     </row>

</xml_diff>